<commit_message>
create workbook with summery & status code
</commit_message>
<xml_diff>
--- a/LogReport.xlsx
+++ b/LogReport.xlsx
@@ -7,6 +7,7 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Summary" sheetId="1" r:id="rId2"/>
+    <x:sheet name="Status Codes" sheetId="2" r:id="rId3"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -16,18 +17,31 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t>Hello</x:t>
+    <x:t>Metric</x:t>
   </x:si>
   <x:si>
-    <x:t>World</x:t>
+    <x:t>Value</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total Hits</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Average RTT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Status Code</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hit Count</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="0" formatCode=""/>
+    <x:numFmt numFmtId="164" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="1">
     <x:font>
@@ -65,13 +79,20 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -370,7 +391,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:B1"/>
+  <x:dimension ref="A1:B3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:2">
@@ -378,6 +399,135 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:2">
+      <x:c r="A2" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>2871061</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:2">
+      <x:c r="A3" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="1">
+        <x:v>278.8791478133</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:B12"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:2">
+      <x:c r="A1" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:2">
+      <x:c r="A2" s="0">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>2766591</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:2">
+      <x:c r="A3" s="0">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
+        <x:v>41071</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:2">
+      <x:c r="A4" s="0">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>47825</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:2">
+      <x:c r="A5" s="0">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>13446</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:2">
+      <x:c r="A6" s="0">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:2">
+      <x:c r="A7" s="0">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>2055</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:2">
+      <x:c r="A8" s="0">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:2">
+      <x:c r="A9" s="0">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:2">
+      <x:c r="A10" s="0">
+        <x:v>504</x:v>
+      </x:c>
+      <x:c r="B10" s="0">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:2">
+      <x:c r="A11" s="0">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="B11" s="0">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:2">
+      <x:c r="A12" s="0">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="B12" s="0">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>